<commit_message>
docs: add Hiatus social summary assets
</commit_message>
<xml_diff>
--- a/docs/plans/assets/module-cutlists/2026-06-25_module-cutlist-and-assignments.xlsx
+++ b/docs/plans/assets/module-cutlists/2026-06-25_module-cutlist-and-assignments.xlsx
@@ -605,6 +605,11 @@
           <t>Electrical | passenger wall / inner | Horizontal</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -658,6 +663,11 @@
           <t>Electrical | passenger wall | Horizontal</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -679,6 +689,11 @@
           <t>Electrical | bulkhead corner | Vertical</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -700,6 +715,11 @@
           <t>Electrical | passenger wall / top | Horizontal</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -721,6 +741,11 @@
           <t>Electrical | top corner | Horizontal</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -742,6 +767,11 @@
           <t>Electrical | bulkhead / driver wall / inner | Vertical</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -763,6 +793,11 @@
           <t>Electrical | passenger wall / top / inner | Horizontal</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -784,6 +819,11 @@
           <t>Electrical | top / inner corner | Horizontal</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -858,6 +898,11 @@
           <t>Electrical | bulkhead / top | Horizontal</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -927,6 +972,11 @@
           <t>Electrical | bulkhead / top / inner | Horizontal</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -1059,6 +1109,11 @@
           <t>Electrical | passenger wall / inner | Vertical</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -1112,6 +1167,11 @@
           <t>Electrical | passenger wall / floor | Horizontal</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -1181,6 +1241,11 @@
           <t>Electrical | passenger wall / inner | Vertical</t>
         </is>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -1419,6 +1484,11 @@
           <t>Electrical | passenger wall / floor / inner | Horizontal</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
@@ -1440,6 +1510,11 @@
           <t>Electrical | bulkhead / floor | Horizontal</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -1566,6 +1641,11 @@
           <t>Electrical | passenger wall | Vertical</t>
         </is>
       </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -1587,6 +1667,11 @@
           <t>Electrical | floor / bottom corner | Horizontal</t>
         </is>
       </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -1624,6 +1709,11 @@
           <t>Electrical | inner / outer corner | Vertical</t>
         </is>
       </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -1645,6 +1735,11 @@
           <t>Electrical | inner corner | Vertical</t>
         </is>
       </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
@@ -1788,6 +1883,11 @@
           <t>Electrical | passenger wall / top | Horizontal</t>
         </is>
       </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -1807,6 +1907,11 @@
       <c r="E69" t="inlineStr">
         <is>
           <t>Electrical | passenger wall / inner | Horizontal</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2582,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O5" s="13" t="n"/>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="6" hidden="1">
       <c r="A6" t="inlineStr">
@@ -2634,7 +2743,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O8" s="13" t="n"/>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2701,7 +2814,11 @@
           <t>Vertical</t>
         </is>
       </c>
-      <c r="O9" s="13" t="n"/>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2768,7 +2885,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O10" s="13" t="n"/>
+      <c r="O10" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2825,7 +2946,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O11" s="13" t="n"/>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2892,7 +3017,11 @@
           <t>Vertical</t>
         </is>
       </c>
-      <c r="O12" s="13" t="n"/>
+      <c r="O12" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2959,7 +3088,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O13" s="13" t="n"/>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3016,7 +3149,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O14" s="13" t="n"/>
+      <c r="O14" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="15" hidden="1">
       <c r="A15" t="inlineStr">
@@ -3230,7 +3367,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O18" s="13" t="n"/>
+      <c r="O18" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="19" hidden="1">
       <c r="A19" t="inlineStr">
@@ -3432,7 +3573,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O22" s="13" t="n"/>
+      <c r="O22" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="23" hidden="1">
       <c r="A23" t="inlineStr">
@@ -3809,7 +3954,11 @@
           <t>Vertical</t>
         </is>
       </c>
-      <c r="O29" s="13" t="n"/>
+      <c r="O29" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="30" hidden="1">
       <c r="A30" t="inlineStr">
@@ -3966,7 +4115,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O32" s="13" t="n"/>
+      <c r="O32" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="33" hidden="1">
       <c r="A33" t="inlineStr">
@@ -4168,7 +4321,11 @@
           <t>Vertical</t>
         </is>
       </c>
-      <c r="O36" s="13" t="n"/>
+      <c r="O36" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="37" hidden="1">
       <c r="A37" t="inlineStr">
@@ -4674,7 +4831,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O46" s="13" t="n"/>
+      <c r="O46" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4731,7 +4892,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O47" s="13" t="n"/>
+      <c r="O47" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="48" hidden="1">
       <c r="A48" t="inlineStr">
@@ -5091,7 +5256,11 @@
           <t>Vertical</t>
         </is>
       </c>
-      <c r="O53" s="13" t="n"/>
+      <c r="O53" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5148,7 +5317,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O54" s="13" t="n"/>
+      <c r="O54" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="55" hidden="1">
       <c r="A55" t="inlineStr">
@@ -5260,7 +5433,11 @@
           <t>Vertical</t>
         </is>
       </c>
-      <c r="O56" s="13" t="n"/>
+      <c r="O56" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5327,7 +5504,11 @@
           <t>Vertical</t>
         </is>
       </c>
-      <c r="O57" s="13" t="n"/>
+      <c r="O57" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="58" hidden="1">
       <c r="A58" t="inlineStr">
@@ -5719,7 +5900,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O65" s="13" t="n"/>
+      <c r="O65" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5776,7 +5961,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O66" s="13" t="n"/>
+      <c r="O66" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="67" hidden="1">
       <c r="A67" t="inlineStr">
@@ -7126,6 +7315,11 @@
           <t>Single-piece row.</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7189,6 +7383,11 @@
           <t>Single-piece row.</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7252,6 +7451,11 @@
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7315,6 +7519,11 @@
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7378,6 +7587,11 @@
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7706,6 +7920,11 @@
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7769,6 +7988,11 @@
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7883,6 +8107,11 @@
       <c r="M15" t="inlineStr">
         <is>
           <t>Single-piece row.</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-26 electrical frame</t>
         </is>
       </c>
     </row>
@@ -9126,7 +9355,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Single-piece row.</t>
+          <t>Single-piece row. | CUT 2026-06-26 electrical frame</t>
         </is>
       </c>
     </row>
@@ -9178,7 +9407,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Single-piece row.</t>
+          <t>Single-piece row. | CUT 2026-06-26 electrical frame</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9459,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Old mapping hinted 2 of 2 identical pieces in this row; any 2 should be interchangeable if the CAD still wants the same count.</t>
+          <t>Old mapping hinted 2 of 2 identical pieces in this row; any 2 should be interchangeable if the CAD still wants the same count. | CUT 2026-06-26 electrical frame</t>
         </is>
       </c>
     </row>
@@ -9282,7 +9511,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Old mapping hinted 2 of 2 identical pieces in this row; any 2 should be interchangeable if the CAD still wants the same count.</t>
+          <t>Old mapping hinted 2 of 2 identical pieces in this row; any 2 should be interchangeable if the CAD still wants the same count. | CUT 2026-06-26 electrical frame</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9563,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Old mapping hinted 3 of 5 identical pieces in this row; any 3 should be interchangeable if the CAD still wants the same count.</t>
+          <t>Old mapping hinted 3 of 5 identical pieces in this row; any 3 should be interchangeable if the CAD still wants the same count. | CUT 2026-06-26 electrical frame</t>
         </is>
       </c>
     </row>
@@ -9386,7 +9615,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Old mapping hinted 2 of 4 identical pieces in this row; any 2 should be interchangeable if the CAD still wants the same count.</t>
+          <t>Old mapping hinted 2 of 4 identical pieces in this row; any 2 should be interchangeable if the CAD still wants the same count. | CUT 2026-06-26 electrical frame</t>
         </is>
       </c>
     </row>
@@ -9438,7 +9667,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Old mapping hinted 1 of 3 identical pieces in this row; any 1 should be interchangeable if the CAD still wants the same count.</t>
+          <t>Old mapping hinted 1 of 3 identical pieces in this row; any 1 should be interchangeable if the CAD still wants the same count. | CUT 2026-06-26 electrical frame</t>
         </is>
       </c>
     </row>
@@ -9490,7 +9719,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Single-piece row.</t>
+          <t>Single-piece row. | CUT 2026-06-26 electrical frame</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tag galley extrusion assignments
</commit_message>
<xml_diff>
--- a/docs/plans/assets/module-cutlists/2026-06-25_module-cutlist-and-assignments.xlsx
+++ b/docs/plans/assets/module-cutlists/2026-06-25_module-cutlist-and-assignments.xlsx
@@ -547,6 +547,11 @@
       <c r="D2" s="3" t="n">
         <v>1270</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -626,6 +631,11 @@
       <c r="D6" s="3" t="n">
         <v>1219.2</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -642,6 +652,11 @@
       <c r="D7" s="3" t="n">
         <v>876.3</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -856,6 +871,11 @@
       <c r="D16" s="3" t="n">
         <v>876.3</v>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -935,6 +955,11 @@
       <c r="D20" s="3" t="n">
         <v>876.3</v>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -951,6 +976,16 @@
       <c r="D21" s="3" t="n">
         <v>254</v>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-29 bench</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -1278,6 +1313,11 @@
       <c r="D38" s="3" t="n">
         <v>850.9</v>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -1357,6 +1397,11 @@
       <c r="D42" s="3" t="n">
         <v>850.9</v>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -1405,6 +1450,11 @@
       <c r="D45" s="3" t="n">
         <v>406.4</v>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -1421,6 +1471,11 @@
       <c r="D46" s="3" t="n">
         <v>812.8</v>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -1463,6 +1518,11 @@
           <t>Bench | top / inner | Horizontal</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-29 bench</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -1774,7 +1834,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Bench</t>
+          <t>Galley</t>
         </is>
       </c>
     </row>
@@ -1846,6 +1906,11 @@
       <c r="D66" s="3" t="n">
         <v>254</v>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
@@ -1862,6 +1927,11 @@
       <c r="D67" s="3" t="n">
         <v>254</v>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -2041,6 +2111,11 @@
       <c r="D76" s="3" t="n">
         <v>355.6</v>
       </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
@@ -2057,6 +2132,11 @@
       <c r="D77" s="3" t="n">
         <v>355.6</v>
       </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
@@ -2073,6 +2153,11 @@
       <c r="D78" s="3" t="n">
         <v>355.6</v>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
@@ -2089,6 +2174,11 @@
       <c r="D79" s="3" t="n">
         <v>355.6</v>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
@@ -2158,6 +2248,11 @@
       <c r="D83" s="3" t="n">
         <v>431.8</v>
       </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
@@ -2174,6 +2269,11 @@
       <c r="D84" s="3" t="n">
         <v>381</v>
       </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
@@ -2206,6 +2306,11 @@
       <c r="D86" s="3" t="n">
         <v>381</v>
       </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
@@ -2222,6 +2327,11 @@
       <c r="D87" s="3" t="n">
         <v>381</v>
       </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
@@ -2238,6 +2348,11 @@
       <c r="D88" s="3" t="n">
         <v>381</v>
       </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
@@ -2254,6 +2369,11 @@
       <c r="D89" s="3" t="n">
         <v>381</v>
       </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
@@ -2269,6 +2389,11 @@
       </c>
       <c r="D90" s="3" t="n">
         <v>381</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2420,10 +2545,18 @@
           <t>R22</t>
         </is>
       </c>
-      <c r="L2" s="13" t="n"/>
+      <c r="L2" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M2" s="13" t="n"/>
       <c r="N2" s="13" t="n"/>
-      <c r="O2" s="13" t="n"/>
+      <c r="O2" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="3" hidden="1">
       <c r="A3" t="inlineStr">
@@ -2628,10 +2761,18 @@
           <t>R31</t>
         </is>
       </c>
-      <c r="L6" s="13" t="n"/>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M6" s="13" t="n"/>
       <c r="N6" s="13" t="n"/>
-      <c r="O6" s="13" t="n"/>
+      <c r="O6" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="7" hidden="1">
       <c r="A7" t="inlineStr">
@@ -2673,10 +2814,18 @@
           <t>R23</t>
         </is>
       </c>
-      <c r="L7" s="13" t="n"/>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M7" s="13" t="n"/>
       <c r="N7" s="13" t="n"/>
-      <c r="O7" s="13" t="n"/>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3240,10 +3389,18 @@
           <t>R23</t>
         </is>
       </c>
-      <c r="L16" s="13" t="n"/>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M16" s="13" t="n"/>
       <c r="N16" s="13" t="n"/>
-      <c r="O16" s="13" t="n"/>
+      <c r="O16" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="17" hidden="1">
       <c r="A17" t="inlineStr">
@@ -3458,10 +3615,18 @@
           <t>R23</t>
         </is>
       </c>
-      <c r="L20" s="13" t="n"/>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M20" s="13" t="n"/>
       <c r="N20" s="13" t="n"/>
-      <c r="O20" s="13" t="n"/>
+      <c r="O20" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="21" hidden="1">
       <c r="A21" t="inlineStr">
@@ -3503,10 +3668,18 @@
           <t>R21</t>
         </is>
       </c>
-      <c r="L21" s="13" t="n"/>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
       <c r="M21" s="13" t="n"/>
       <c r="N21" s="13" t="n"/>
-      <c r="O21" s="13" t="n"/>
+      <c r="O21" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-29 bench</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4412,10 +4585,18 @@
           <t>R32</t>
         </is>
       </c>
-      <c r="L38" s="13" t="n"/>
+      <c r="L38" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M38" s="13" t="n"/>
       <c r="N38" s="13" t="n"/>
-      <c r="O38" s="13" t="n"/>
+      <c r="O38" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="39" hidden="1">
       <c r="A39" t="inlineStr">
@@ -4518,10 +4699,18 @@
           <t>R32</t>
         </is>
       </c>
-      <c r="L40" s="13" t="n"/>
+      <c r="L40" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M40" s="13" t="n"/>
       <c r="N40" s="13" t="n"/>
-      <c r="O40" s="13" t="n"/>
+      <c r="O40" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="41" hidden="1">
       <c r="A41" t="inlineStr">
@@ -4653,10 +4842,18 @@
           <t>R25</t>
         </is>
       </c>
-      <c r="L43" s="13" t="n"/>
+      <c r="L43" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M43" s="13" t="n"/>
       <c r="N43" s="13" t="n"/>
-      <c r="O43" s="13" t="n"/>
+      <c r="O43" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="44" hidden="1">
       <c r="A44" t="inlineStr">
@@ -4774,7 +4971,11 @@
           <t>Horizontal</t>
         </is>
       </c>
-      <c r="O45" s="13" t="n"/>
+      <c r="O45" s="13" t="inlineStr">
+        <is>
+          <t>CUT 2026-06-29 bench</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5597,12 +5798,16 @@
       </c>
       <c r="L59" s="13" t="inlineStr">
         <is>
-          <t>Bench</t>
+          <t>Galley</t>
         </is>
       </c>
       <c r="M59" s="13" t="n"/>
       <c r="N59" s="13" t="n"/>
-      <c r="O59" s="13" t="n"/>
+      <c r="O59" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G; reassigned from Bench</t>
+        </is>
+      </c>
     </row>
     <row r="60" hidden="1">
       <c r="A60" t="inlineStr">
@@ -5795,10 +6000,18 @@
           <t>R21</t>
         </is>
       </c>
-      <c r="L63" s="13" t="n"/>
+      <c r="L63" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M63" s="13" t="n"/>
       <c r="N63" s="13" t="n"/>
-      <c r="O63" s="13" t="n"/>
+      <c r="O63" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="64" hidden="1">
       <c r="A64" t="inlineStr">
@@ -5840,10 +6053,18 @@
           <t>R21</t>
         </is>
       </c>
-      <c r="L64" s="13" t="n"/>
+      <c r="L64" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M64" s="13" t="n"/>
       <c r="N64" s="13" t="n"/>
-      <c r="O64" s="13" t="n"/>
+      <c r="O64" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6317,10 +6538,18 @@
           <t>R18</t>
         </is>
       </c>
-      <c r="L73" s="13" t="n"/>
+      <c r="L73" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M73" s="13" t="n"/>
       <c r="N73" s="13" t="n"/>
-      <c r="O73" s="13" t="n"/>
+      <c r="O73" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="74" hidden="1">
       <c r="A74" t="inlineStr">
@@ -6362,10 +6591,18 @@
           <t>R18</t>
         </is>
       </c>
-      <c r="L74" s="13" t="n"/>
+      <c r="L74" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M74" s="13" t="n"/>
       <c r="N74" s="13" t="n"/>
-      <c r="O74" s="13" t="n"/>
+      <c r="O74" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="75" hidden="1">
       <c r="A75" t="inlineStr">
@@ -6407,10 +6644,18 @@
           <t>R18</t>
         </is>
       </c>
-      <c r="L75" s="13" t="n"/>
+      <c r="L75" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M75" s="13" t="n"/>
       <c r="N75" s="13" t="n"/>
-      <c r="O75" s="13" t="n"/>
+      <c r="O75" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="76" hidden="1">
       <c r="A76" t="inlineStr">
@@ -6452,10 +6697,18 @@
           <t>R18</t>
         </is>
       </c>
-      <c r="L76" s="13" t="n"/>
+      <c r="L76" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M76" s="13" t="n"/>
       <c r="N76" s="13" t="n"/>
-      <c r="O76" s="13" t="n"/>
+      <c r="O76" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="77" hidden="1">
       <c r="A77" t="inlineStr">
@@ -6587,10 +6840,18 @@
           <t>R19</t>
         </is>
       </c>
-      <c r="L79" s="13" t="n"/>
+      <c r="L79" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M79" s="13" t="n"/>
       <c r="N79" s="13" t="n"/>
-      <c r="O79" s="13" t="n"/>
+      <c r="O79" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="80" hidden="1">
       <c r="A80" t="inlineStr">
@@ -6677,10 +6938,18 @@
           <t>R19</t>
         </is>
       </c>
-      <c r="L81" s="13" t="n"/>
+      <c r="L81" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M81" s="13" t="n"/>
       <c r="N81" s="13" t="n"/>
-      <c r="O81" s="13" t="n"/>
+      <c r="O81" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="82" hidden="1">
       <c r="A82" t="inlineStr">
@@ -6722,10 +6991,18 @@
           <t>R19</t>
         </is>
       </c>
-      <c r="L82" s="13" t="n"/>
+      <c r="L82" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M82" s="13" t="n"/>
       <c r="N82" s="13" t="n"/>
-      <c r="O82" s="13" t="n"/>
+      <c r="O82" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="83" hidden="1">
       <c r="A83" t="inlineStr">
@@ -6767,10 +7044,18 @@
           <t>R19</t>
         </is>
       </c>
-      <c r="L83" s="13" t="n"/>
+      <c r="L83" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M83" s="13" t="n"/>
       <c r="N83" s="13" t="n"/>
-      <c r="O83" s="13" t="n"/>
+      <c r="O83" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="84" hidden="1">
       <c r="A84" t="inlineStr">
@@ -6812,10 +7097,18 @@
           <t>R19</t>
         </is>
       </c>
-      <c r="L84" s="13" t="n"/>
+      <c r="L84" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M84" s="13" t="n"/>
       <c r="N84" s="13" t="n"/>
-      <c r="O84" s="13" t="n"/>
+      <c r="O84" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="85" hidden="1">
       <c r="A85" t="inlineStr">
@@ -6857,10 +7150,18 @@
           <t>R19</t>
         </is>
       </c>
-      <c r="L85" s="13" t="n"/>
+      <c r="L85" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M85" s="13" t="n"/>
       <c r="N85" s="13" t="n"/>
-      <c r="O85" s="13" t="n"/>
+      <c r="O85" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="86" hidden="1">
       <c r="A86" t="inlineStr">
@@ -7024,10 +7325,18 @@
           <t>R33 R34</t>
         </is>
       </c>
-      <c r="L88" s="13" t="n"/>
+      <c r="L88" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M88" s="13" t="n"/>
       <c r="N88" s="13" t="n"/>
-      <c r="O88" s="13" t="n"/>
+      <c r="O88" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
     <row r="89" hidden="1">
       <c r="A89" t="inlineStr">
@@ -7130,10 +7439,18 @@
           <t>R20 R35</t>
         </is>
       </c>
-      <c r="L90" s="13" t="n"/>
+      <c r="L90" s="13" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
       <c r="M90" s="13" t="n"/>
       <c r="N90" s="13" t="n"/>
-      <c r="O90" s="13" t="n"/>
+      <c r="O90" s="13" t="inlineStr">
+        <is>
+          <t>Galley CSV 2026-07-02; mark G</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O90">
@@ -7302,12 +7619,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Electrical panel frame</t>
+          <t>Electrical: 1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>bottom left</t>
+          <t>passenger wall / floor: 1</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -7370,12 +7687,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Electrical panel frame</t>
+          <t>Electrical: 1</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>rear vertical inner</t>
+          <t>passenger wall / inner: 1</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -7438,12 +7755,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Electrical panel frame</t>
+          <t>Electrical: 2</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>bulkhead vertical</t>
+          <t>bulkhead / driver wall / inner: 1; bulkhead corner: 1</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -7506,12 +7823,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Electrical panel frame</t>
+          <t>Electrical: 2</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>top</t>
+          <t>passenger wall / top: 1; passenger wall / top / inner: 1</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -7574,12 +7891,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Electrical panel frame</t>
+          <t>Electrical: 3</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>rear vertical</t>
+          <t>inner / outer corner: 1; inner corner: 1; passenger wall: 1</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -7691,7 +8008,17 @@
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Bench: 1; Electrical: 2</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>floor: 1; top / inner corner: 1; top corner: 1</t>
+        </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -7744,7 +8071,17 @@
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Electrical: 1</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>floor / bottom corner: 1</t>
+        </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -7850,7 +8187,17 @@
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Electrical: 2</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>passenger wall / floor / inner: 1; passenger wall / inner: 1</t>
+        </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -7903,16 +8250,16 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Electrical panel frame</t>
+          <t>Electrical: 4</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>top horizontal</t>
+          <t>bulkhead / floor: 1; bulkhead / top: 1; bulkhead / top / inner: 1; passenger wall / top: 1</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -7975,12 +8322,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Electrical panel frame</t>
+          <t>Electrical: 1</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>rear vertical inner corner</t>
+          <t>passenger wall / inner: 1</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -8039,7 +8386,17 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Electrical: 1</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>passenger wall / inner: 1</t>
+        </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -8096,12 +8453,12 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Electrical panel frame</t>
+          <t>Electrical: 1</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>rear horizontal mid</t>
+          <t>passenger wall: 1</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -8266,7 +8623,17 @@
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Bench: 4</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>driver wall / floor: 1; driver wall / floor / inner: 1; driver wall / upper: 1; driver wall / upper / inner: 1</t>
+        </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -8319,11 +8686,26 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Bench: 3; Galley: 4</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>bulkhead / floor: 1; floor: 1; upper: 1</t>
+        </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Galley assigned 4 of 7 unassigned pieces from owner CSV 2026-07-02; existing Bench pieces preserved.</t>
         </is>
       </c>
     </row>
@@ -8372,11 +8754,26 @@
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Bench: 2; Galley: 6</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>bulkhead: 1; bulkhead / driver wall corner: 1</t>
+        </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Galley assigned 6 of 8 unassigned pieces from owner CSV 2026-07-02; existing Bench pieces preserved.</t>
         </is>
       </c>
     </row>
@@ -8425,7 +8822,17 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Bench: 1</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>bulkhead: 1</t>
+        </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -8478,11 +8885,26 @@
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Bench: 2; Galley: 2</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>driver wall: 1</t>
+        </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Galley assigned 2 of 4 unassigned pieces from owner CSV 2026-07-02; existing Bench pieces preserved.</t>
         </is>
       </c>
     </row>
@@ -8531,11 +8953,21 @@
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Galley: 1</t>
+        </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>Single-piece row.</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Galley assigned 1 of 1 from owner CSV 2026-07-02.</t>
         </is>
       </c>
     </row>
@@ -8584,11 +9016,21 @@
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Galley: 3</t>
+        </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Galley assigned 3 of 3 from owner CSV 2026-07-02.</t>
         </is>
       </c>
     </row>
@@ -8637,11 +9079,21 @@
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Galley: 1</t>
+        </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
           <t>Single-piece row.</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Galley assigned 1 of 1 from owner CSV 2026-07-02; reassigned from prior Bench tag.</t>
         </is>
       </c>
     </row>
@@ -8690,11 +9142,21 @@
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Galley: 1</t>
+        </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
           <t>Single-piece row.</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Galley assigned 1 of 1 from owner CSV 2026-07-02.</t>
         </is>
       </c>
     </row>
@@ -8743,7 +9205,17 @@
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Bench: 1</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>top / inner: 1</t>
+        </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -8796,7 +9268,17 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Bench: 2</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>driver wall / upper: 1; passenger wall / inner: 1</t>
+        </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -8849,7 +9331,17 @@
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Bench: 2</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>bulkhead / lower: 1; bulkhead / upper: 1</t>
+        </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -8902,7 +9394,17 @@
         </is>
       </c>
       <c r="J30" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Bench: 1</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>driver wall / inner: 1</t>
+        </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -9008,11 +9510,21 @@
         </is>
       </c>
       <c r="J32" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Galley: 1</t>
+        </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
           <t>Single-piece row.</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Galley assigned 1 of 1 from owner CSV 2026-07-02.</t>
         </is>
       </c>
     </row>
@@ -9061,11 +9573,21 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Galley: 2</t>
+        </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Galley assigned 2 of 2 from owner CSV 2026-07-02.</t>
         </is>
       </c>
     </row>
@@ -9114,7 +9636,17 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Bench: 2</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>driver wall: 1; driver wall / inner: 1</t>
+        </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -9167,11 +9699,21 @@
         </is>
       </c>
       <c r="J35" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Galley: 1</t>
+        </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
           <t>Single-piece row.</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Galley assigned 1 of 1 smooth-stock row from owner CSV 2026-07-02.</t>
         </is>
       </c>
     </row>
@@ -9220,11 +9762,21 @@
         </is>
       </c>
       <c r="J36" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Galley: 1</t>
+        </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
           <t>Single-piece row.</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Galley assigned 1 of 1 smooth-stock row from owner CSV 2026-07-02.</t>
         </is>
       </c>
     </row>
@@ -9735,7 +10287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9762,7 +10314,7 @@
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Electrical; Bench; blank = not assigned yet</t>
+          <t>Electrical; Bench; Galley; blank = not assigned yet</t>
         </is>
       </c>
     </row>
@@ -9851,81 +10403,81 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="n"/>
-      <c r="B11" s="15" t="n"/>
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Galley</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>Orientation</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>Assigned rows</t>
-        </is>
-      </c>
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Horizontal</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="n">
-        <v>28</v>
+          <t>Orientation</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>Assigned rows</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
+          <t>Horizontal</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
           <t>Vertical</t>
         </is>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B15" s="15" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="15" t="n"/>
-      <c r="B15" s="15" t="n"/>
-    </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>Assigned rows</t>
-        </is>
-      </c>
+      <c r="A16" s="15" t="n"/>
+      <c r="B16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>passenger wall / inner</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="n">
-        <v>5</v>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Assigned rows</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>passenger wall / inner</t>
         </is>
       </c>
       <c r="B18" s="15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>passenger wall</t>
+          <t>bulkhead</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
@@ -9935,7 +10487,7 @@
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>passenger wall / top</t>
+          <t>bulkhead / floor</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -9955,7 +10507,7 @@
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>driver wall / upper</t>
+          <t>driver wall / inner</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -9965,7 +10517,7 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / floor</t>
+          <t>driver wall / upper</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -9975,7 +10527,7 @@
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>driver wall / inner</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -9985,7 +10537,7 @@
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>bulkhead</t>
+          <t>passenger wall</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -9995,17 +10547,17 @@
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>bulkhead corner</t>
+          <t>passenger wall / top</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>top corner</t>
+          <t>bulkhead / driver wall / inner</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
@@ -10015,7 +10567,7 @@
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / driver wall / inner</t>
+          <t>bulkhead / driver wall corner</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -10025,7 +10577,7 @@
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>passenger wall / top / inner</t>
+          <t>bulkhead / lower</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -10035,7 +10587,7 @@
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>top / inner corner</t>
+          <t>bulkhead / top</t>
         </is>
       </c>
       <c r="B30" s="15" t="n">
@@ -10045,7 +10597,7 @@
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / top</t>
+          <t>bulkhead / top / inner</t>
         </is>
       </c>
       <c r="B31" s="15" t="n">
@@ -10055,7 +10607,7 @@
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / top / inner</t>
+          <t>bulkhead / upper</t>
         </is>
       </c>
       <c r="B32" s="15" t="n">
@@ -10065,7 +10617,7 @@
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / upper</t>
+          <t>bulkhead corner</t>
         </is>
       </c>
       <c r="B33" s="15" t="n">
@@ -10075,7 +10627,7 @@
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>upper</t>
+          <t>driver wall / floor</t>
         </is>
       </c>
       <c r="B34" s="15" t="n">
@@ -10085,7 +10637,7 @@
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / lower</t>
+          <t>driver wall / floor / inner</t>
         </is>
       </c>
       <c r="B35" s="15" t="n">
@@ -10095,7 +10647,7 @@
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>passenger wall / floor</t>
+          <t>driver wall / upper / inner</t>
         </is>
       </c>
       <c r="B36" s="15" t="n">
@@ -10105,7 +10657,7 @@
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>top / inner</t>
+          <t>floor / bottom corner</t>
         </is>
       </c>
       <c r="B37" s="15" t="n">
@@ -10115,7 +10667,7 @@
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
         <is>
-          <t>passenger wall / floor / inner</t>
+          <t>inner / outer corner</t>
         </is>
       </c>
       <c r="B38" s="15" t="n">
@@ -10125,7 +10677,7 @@
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>driver wall / floor / inner</t>
+          <t>inner corner</t>
         </is>
       </c>
       <c r="B39" s="15" t="n">
@@ -10135,7 +10687,7 @@
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t>driver wall / upper / inner</t>
+          <t>passenger wall / floor</t>
         </is>
       </c>
       <c r="B40" s="15" t="n">
@@ -10145,7 +10697,7 @@
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>driver wall / floor</t>
+          <t>passenger wall / floor / inner</t>
         </is>
       </c>
       <c r="B41" s="15" t="n">
@@ -10155,7 +10707,7 @@
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>floor / bottom corner</t>
+          <t>passenger wall / top / inner</t>
         </is>
       </c>
       <c r="B42" s="15" t="n">
@@ -10165,7 +10717,7 @@
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>inner / outer corner</t>
+          <t>top / inner</t>
         </is>
       </c>
       <c r="B43" s="15" t="n">
@@ -10175,7 +10727,7 @@
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
         <is>
-          <t>inner corner</t>
+          <t>top / inner corner</t>
         </is>
       </c>
       <c r="B44" s="15" t="n">
@@ -10185,10 +10737,20 @@
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / driver wall corner</t>
+          <t>top corner</t>
         </is>
       </c>
       <c r="B45" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tag desk extrusion assignments
</commit_message>
<xml_diff>
--- a/docs/plans/assets/module-cutlists/2026-06-25_module-cutlist-and-assignments.xlsx
+++ b/docs/plans/assets/module-cutlists/2026-06-25_module-cutlist-and-assignments.xlsx
@@ -8,16 +8,18 @@
   <sheets>
     <sheet name="garage_final_cutlist" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="piece_assignment" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="source_row_pools" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="electrical_seed" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="assignment_legend" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="desk_shop_list" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="source_row_pools" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="electrical_seed" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="assignment_legend" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'garage_final_cutlist'!$A$1:$F$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'piece_assignment'!$A$1:$O$90</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'source_row_pools'!$A$1:$N$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'electrical_seed'!$A$1:$J$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'assignment_legend'!$A$1:$B$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'desk_shop_list'!$A$1:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'source_row_pools'!$A$1:$N$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'electrical_seed'!$A$1:$J$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'assignment_legend'!$A$1:$B$45</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,11 +27,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0##"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +54,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -99,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -123,6 +129,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -589,6 +600,11 @@
       <c r="D4" s="3" t="n">
         <v>419.1</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -855,6 +871,11 @@
       <c r="D15" s="3" t="n">
         <v>1143</v>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -939,6 +960,11 @@
       <c r="D19" s="3" t="n">
         <v>1143</v>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1049,6 +1075,11 @@
       <c r="D24" s="3" t="n">
         <v>558.8</v>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -1065,6 +1096,11 @@
       <c r="D25" s="3" t="n">
         <v>469.9</v>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -1123,6 +1159,11 @@
       <c r="D28" s="3" t="n">
         <v>469.9</v>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -1165,6 +1206,11 @@
       <c r="D30" s="3" t="n">
         <v>457.2</v>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -1181,6 +1227,11 @@
       <c r="D31" s="3" t="n">
         <v>939.8</v>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -1223,6 +1274,11 @@
       <c r="D33" s="3" t="n">
         <v>558.8</v>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -1239,6 +1295,11 @@
       <c r="D34" s="3" t="n">
         <v>914.4</v>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -1255,6 +1316,11 @@
       <c r="D35" s="3" t="n">
         <v>558.8</v>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -1297,6 +1363,11 @@
       <c r="D37" s="3" t="n">
         <v>419.1</v>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -1418,6 +1489,11 @@
       <c r="D43" s="3" t="n">
         <v>558.8</v>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -1434,6 +1510,11 @@
       <c r="D44" s="3" t="n">
         <v>558.8</v>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -1748,6 +1829,11 @@
       <c r="D58" s="3" t="n">
         <v>419.1</v>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
@@ -1816,6 +1902,11 @@
       <c r="D61" s="3" t="n">
         <v>558.8</v>
       </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
@@ -1853,6 +1944,11 @@
       <c r="D63" s="3" t="n">
         <v>685.8</v>
       </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
@@ -1869,6 +1965,11 @@
       <c r="D64" s="3" t="n">
         <v>685.8</v>
       </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -2000,6 +2101,11 @@
       <c r="D70" s="3" t="n">
         <v>533.4</v>
       </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
@@ -2016,6 +2122,11 @@
       <c r="D71" s="3" t="n">
         <v>533.4</v>
       </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -2074,6 +2185,11 @@
       <c r="D74" s="3" t="n">
         <v>558.8</v>
       </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -2195,6 +2311,11 @@
       <c r="D80" s="3" t="n">
         <v>558.8</v>
       </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
@@ -2211,6 +2332,11 @@
       <c r="D81" s="3" t="n">
         <v>558.8</v>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
@@ -2289,6 +2415,11 @@
       </c>
       <c r="D85" s="3" t="n">
         <v>457.2</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -2655,7 +2786,11 @@
           <t>R30</t>
         </is>
       </c>
-      <c r="L4" s="13" t="n"/>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M4" s="13" t="n"/>
       <c r="N4" s="13" t="n"/>
       <c r="O4" s="13" t="n"/>
@@ -3344,7 +3479,11 @@
           <t>R16</t>
         </is>
       </c>
-      <c r="L15" s="13" t="n"/>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M15" s="13" t="n"/>
       <c r="N15" s="13" t="n"/>
       <c r="O15" s="13" t="n"/>
@@ -3570,7 +3709,11 @@
           <t>R16</t>
         </is>
       </c>
-      <c r="L19" s="13" t="n"/>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M19" s="13" t="n"/>
       <c r="N19" s="13" t="n"/>
       <c r="O19" s="13" t="n"/>
@@ -3849,7 +3992,11 @@
           <t>R07</t>
         </is>
       </c>
-      <c r="L24" s="13" t="n"/>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M24" s="13" t="n"/>
       <c r="N24" s="13" t="n"/>
       <c r="O24" s="13" t="n"/>
@@ -3894,7 +4041,11 @@
           <t>R15</t>
         </is>
       </c>
-      <c r="L25" s="13" t="n"/>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M25" s="13" t="n"/>
       <c r="N25" s="13" t="n"/>
       <c r="O25" s="13" t="n"/>
@@ -4057,7 +4208,11 @@
           <t>R15</t>
         </is>
       </c>
-      <c r="L28" s="13" t="n"/>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M28" s="13" t="n"/>
       <c r="N28" s="13" t="n"/>
       <c r="O28" s="13" t="n"/>
@@ -4173,7 +4328,11 @@
           <t>R12</t>
         </is>
       </c>
-      <c r="L30" s="13" t="n"/>
+      <c r="L30" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M30" s="13" t="n"/>
       <c r="N30" s="13" t="n"/>
       <c r="O30" s="13" t="n"/>
@@ -4218,7 +4377,11 @@
           <t>R06</t>
         </is>
       </c>
-      <c r="L31" s="13" t="n"/>
+      <c r="L31" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M31" s="13" t="n"/>
       <c r="N31" s="13" t="n"/>
       <c r="O31" s="13" t="n"/>
@@ -4334,7 +4497,11 @@
           <t>R07</t>
         </is>
       </c>
-      <c r="L33" s="13" t="n"/>
+      <c r="L33" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M33" s="13" t="n"/>
       <c r="N33" s="13" t="n"/>
       <c r="O33" s="13" t="n"/>
@@ -4379,7 +4546,11 @@
           <t>R09</t>
         </is>
       </c>
-      <c r="L34" s="13" t="n"/>
+      <c r="L34" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M34" s="13" t="n"/>
       <c r="N34" s="13" t="n"/>
       <c r="O34" s="13" t="n"/>
@@ -4424,7 +4595,11 @@
           <t>R07</t>
         </is>
       </c>
-      <c r="L35" s="13" t="n"/>
+      <c r="L35" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M35" s="13" t="n"/>
       <c r="N35" s="13" t="n"/>
       <c r="O35" s="13" t="n"/>
@@ -4540,7 +4715,11 @@
           <t>R30</t>
         </is>
       </c>
-      <c r="L37" s="13" t="n"/>
+      <c r="L37" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M37" s="13" t="n"/>
       <c r="N37" s="13" t="n"/>
       <c r="O37" s="13" t="n"/>
@@ -4752,7 +4931,11 @@
           <t>R07</t>
         </is>
       </c>
-      <c r="L41" s="13" t="n"/>
+      <c r="L41" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M41" s="13" t="n"/>
       <c r="N41" s="13" t="n"/>
       <c r="O41" s="13" t="n"/>
@@ -4797,7 +4980,11 @@
           <t>R07</t>
         </is>
       </c>
-      <c r="L42" s="13" t="n"/>
+      <c r="L42" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M42" s="13" t="n"/>
       <c r="N42" s="13" t="n"/>
       <c r="O42" s="13" t="n"/>
@@ -5564,7 +5751,11 @@
           <t>R30</t>
         </is>
       </c>
-      <c r="L55" s="13" t="n"/>
+      <c r="L55" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M55" s="13" t="n"/>
       <c r="N55" s="13" t="n"/>
       <c r="O55" s="13" t="n"/>
@@ -5751,7 +5942,11 @@
           <t>R07</t>
         </is>
       </c>
-      <c r="L58" s="13" t="n"/>
+      <c r="L58" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M58" s="13" t="n"/>
       <c r="N58" s="13" t="n"/>
       <c r="O58" s="13" t="n"/>
@@ -5849,7 +6044,11 @@
           <t>R05</t>
         </is>
       </c>
-      <c r="L60" s="13" t="n"/>
+      <c r="L60" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M60" s="13" t="n"/>
       <c r="N60" s="13" t="n"/>
       <c r="O60" s="13" t="n"/>
@@ -5894,7 +6093,11 @@
           <t>R05</t>
         </is>
       </c>
-      <c r="L61" s="13" t="n"/>
+      <c r="L61" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M61" s="13" t="n"/>
       <c r="N61" s="13" t="n"/>
       <c r="O61" s="13" t="n"/>
@@ -6228,7 +6431,11 @@
           <t>R08</t>
         </is>
       </c>
-      <c r="L67" s="13" t="n"/>
+      <c r="L67" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M67" s="13" t="n"/>
       <c r="N67" s="13" t="n"/>
       <c r="O67" s="13" t="n"/>
@@ -6273,7 +6480,11 @@
           <t>R08</t>
         </is>
       </c>
-      <c r="L68" s="13" t="n"/>
+      <c r="L68" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M68" s="13" t="n"/>
       <c r="N68" s="13" t="n"/>
       <c r="O68" s="13" t="n"/>
@@ -6432,7 +6643,11 @@
           <t>R07</t>
         </is>
       </c>
-      <c r="L71" s="13" t="n"/>
+      <c r="L71" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M71" s="13" t="n"/>
       <c r="N71" s="13" t="n"/>
       <c r="O71" s="13" t="n"/>
@@ -6750,7 +6965,11 @@
           <t>R07</t>
         </is>
       </c>
-      <c r="L77" s="13" t="n"/>
+      <c r="L77" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M77" s="13" t="n"/>
       <c r="N77" s="13" t="n"/>
       <c r="O77" s="13" t="n"/>
@@ -6795,7 +7014,11 @@
           <t>R07</t>
         </is>
       </c>
-      <c r="L78" s="13" t="n"/>
+      <c r="L78" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M78" s="13" t="n"/>
       <c r="N78" s="13" t="n"/>
       <c r="O78" s="13" t="n"/>
@@ -6893,7 +7116,11 @@
           <t>R12</t>
         </is>
       </c>
-      <c r="L80" s="13" t="n"/>
+      <c r="L80" s="13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
       <c r="M80" s="13" t="n"/>
       <c r="N80" s="13" t="n"/>
       <c r="O80" s="13" t="n"/>
@@ -7480,6 +7707,1286 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>cut_id</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>planned_stick</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>cut_order</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>source_row</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>piece_id</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>piece_length_in</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>piece_length_mm</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>module</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>shop_note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1010-01</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>R30</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>R30-01</t>
+        </is>
+      </c>
+      <c r="F2" s="16" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1010-05</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>R16-01</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>1143</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>6-1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1010-06</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>R16-02</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>1143</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>7-2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1010-07</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>R07-04</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7-3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1010-07</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>R15-01</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>469.9</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>8-2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1010-08</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>R15-02</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>469.9</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>8-4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1010-08</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>R12-02</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>457.2</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9-1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1010-09</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>R06</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>R06-01</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>939.8</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>9-3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1010-09</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>R07-05</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>10-1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1010-10</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>R09</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>R09-01</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>914.4</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>10-2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1010-10</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>R07-06</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>10-4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1010-10</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>R30</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>R30-02</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12-2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1010-12</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>R07-07</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>12-3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1010-12</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>R07-08</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>15-4</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1010-15</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>R30</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>R30-03</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>16-3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1010-16</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>R07-09</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>17-1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1010-17</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>R05</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>R05-04</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>685.8</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>17-2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1010-17</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>R05</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>R05-05</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>685.8</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>18-2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1010-18</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>R08</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>R08-02</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>533.4</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>18-3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1010-18</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>R08</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>R08-03</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>533.4</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>19-1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1010-19</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>R07-12</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>20-1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1010-20</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>R07-10</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>20-2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1010-20</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>R07-11</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>21-1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1010-21</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>R12-03</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>457.2</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Mark D / Desk remaining pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>Grouped by source row / length</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>source_row</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>qty</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>piece_length_in</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>piece_length_mm</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>cut_ids</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>1143</v>
+      </c>
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>5-1 6-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>R06</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>939.8</v>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>9-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>R09</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>914.4</v>
+      </c>
+      <c r="E32" s="18" t="inlineStr">
+        <is>
+          <t>10-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>R05</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>685.8</v>
+      </c>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>17-1 17-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>9</v>
+      </c>
+      <c r="C34" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="E34" s="18" t="inlineStr">
+        <is>
+          <t>7-2 9-3 10-2 12-2 12-3 16-3 19-1 20-1 20-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>R08</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>533.4</v>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>18-2 18-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" s="16" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>469.9</v>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>7-3 8-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>457.2</v>
+      </c>
+      <c r="E37" s="18" t="inlineStr">
+        <is>
+          <t>8-4 21-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>R30</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C38" s="16" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>1-3 10-4 15-4</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I25"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7494,6 +9001,7 @@
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="12"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
     <col width="55" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
   </cols>
@@ -7887,11 +9395,11 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Electrical: 3</t>
+          <t>Desk: 2; Electrical: 3</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -7906,7 +9414,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>CUT 2026-06-26 electrical frame</t>
+          <t>CUT 2026-06-26 electrical frame | Desk assigned 2026-07-04 from remaining unassigned pool after Bench/Galley/Electrical tie-ins.</t>
         </is>
       </c>
     </row>
@@ -7955,11 +9463,21 @@
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Desk: 1</t>
+        </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>Single-piece row.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Desk assigned 2026-07-04 from remaining unassigned pool after Bench/Galley/Electrical tie-ins.</t>
         </is>
       </c>
     </row>
@@ -8008,11 +9526,11 @@
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Bench: 1; Electrical: 2</t>
+          <t>Bench: 1; Desk: 9; Electrical: 2</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -8023,6 +9541,11 @@
       <c r="M8" t="inlineStr">
         <is>
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Desk assigned 2026-07-04 from remaining unassigned pool after Bench/Galley/Electrical tie-ins.</t>
         </is>
       </c>
     </row>
@@ -8071,11 +9594,11 @@
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Electrical: 1</t>
+          <t>Desk: 2; Electrical: 1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -8086,6 +9609,11 @@
       <c r="M9" t="inlineStr">
         <is>
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Desk assigned 2026-07-04 from remaining unassigned pool after Bench/Galley/Electrical tie-ins.</t>
         </is>
       </c>
     </row>
@@ -8134,11 +9662,21 @@
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Desk: 1</t>
+        </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>Single-piece row.</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Desk assigned 2026-07-04 from remaining unassigned pool after Bench/Galley/Electrical tie-ins.</t>
         </is>
       </c>
     </row>
@@ -8318,11 +9856,11 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Electrical: 1</t>
+          <t>Desk: 2; Electrical: 1</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -8337,7 +9875,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>CUT 2026-06-26 electrical frame</t>
+          <t>CUT 2026-06-26 electrical frame | Desk assigned 2026-07-04 from remaining unassigned pool after Bench/Galley/Electrical tie-ins.</t>
         </is>
       </c>
     </row>
@@ -8517,11 +10055,21 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Desk: 2</t>
+        </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Desk assigned 2026-07-04 from remaining unassigned pool after Bench/Galley/Electrical tie-ins.</t>
         </is>
       </c>
     </row>
@@ -8570,11 +10118,21 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Desk: 2</t>
+        </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Desk assigned 2026-07-04 from remaining unassigned pool after Bench/Galley/Electrical tie-ins.</t>
         </is>
       </c>
     </row>
@@ -9457,11 +11015,21 @@
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Desk: 3</t>
+        </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
           <t>Any piece in this row is interchangeable once you know this row belongs to the module.</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Desk assigned 2026-07-04 from remaining unassigned pool after Bench/Galley/Electrical tie-ins.</t>
         </is>
       </c>
     </row>
@@ -9786,7 +11354,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10281,13 +11849,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10314,7 +11882,7 @@
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Electrical; Bench; Galley; blank = not assigned yet</t>
+          <t>Electrical; Bench; Galley; Desk; blank = not assigned/uncertain</t>
         </is>
       </c>
     </row>
@@ -10395,99 +11963,99 @@
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Desk</t>
         </is>
       </c>
       <c r="B10" s="15" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
           <t>Galley</t>
         </is>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B12" s="15" t="n">
         <v>23</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="15" t="n"/>
-      <c r="B12" s="15" t="n"/>
-    </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>Orientation</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>Assigned rows</t>
-        </is>
-      </c>
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>Horizontal</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="n">
-        <v>28</v>
+          <t>Orientation</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Assigned rows</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
+          <t>Horizontal</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
           <t>Vertical</t>
         </is>
       </c>
-      <c r="B15" s="15" t="n">
+      <c r="B16" s="15" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="15" t="n"/>
-      <c r="B16" s="15" t="n"/>
-    </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="inlineStr">
-        <is>
-          <t>Assigned rows</t>
-        </is>
-      </c>
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>passenger wall / inner</t>
-        </is>
-      </c>
-      <c r="B18" s="15" t="n">
-        <v>5</v>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Assigned rows</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>bulkhead</t>
+          <t>passenger wall / inner</t>
         </is>
       </c>
       <c r="B19" s="15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / floor</t>
+          <t>bulkhead</t>
         </is>
       </c>
       <c r="B20" s="15" t="n">
@@ -10497,7 +12065,7 @@
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>driver wall</t>
+          <t>bulkhead / floor</t>
         </is>
       </c>
       <c r="B21" s="15" t="n">
@@ -10507,7 +12075,7 @@
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>driver wall / inner</t>
+          <t>driver wall</t>
         </is>
       </c>
       <c r="B22" s="15" t="n">
@@ -10517,7 +12085,7 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>driver wall / upper</t>
+          <t>driver wall / inner</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
@@ -10527,7 +12095,7 @@
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>driver wall / upper</t>
         </is>
       </c>
       <c r="B24" s="15" t="n">
@@ -10537,7 +12105,7 @@
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>passenger wall</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="B25" s="15" t="n">
@@ -10547,7 +12115,7 @@
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>passenger wall / top</t>
+          <t>passenger wall</t>
         </is>
       </c>
       <c r="B26" s="15" t="n">
@@ -10557,17 +12125,17 @@
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / driver wall / inner</t>
+          <t>passenger wall / top</t>
         </is>
       </c>
       <c r="B27" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / driver wall corner</t>
+          <t>bulkhead / driver wall / inner</t>
         </is>
       </c>
       <c r="B28" s="15" t="n">
@@ -10577,7 +12145,7 @@
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / lower</t>
+          <t>bulkhead / driver wall corner</t>
         </is>
       </c>
       <c r="B29" s="15" t="n">
@@ -10587,7 +12155,7 @@
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / top</t>
+          <t>bulkhead / lower</t>
         </is>
       </c>
       <c r="B30" s="15" t="n">
@@ -10597,7 +12165,7 @@
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / top / inner</t>
+          <t>bulkhead / top</t>
         </is>
       </c>
       <c r="B31" s="15" t="n">
@@ -10607,7 +12175,7 @@
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>bulkhead / upper</t>
+          <t>bulkhead / top / inner</t>
         </is>
       </c>
       <c r="B32" s="15" t="n">
@@ -10617,7 +12185,7 @@
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>bulkhead corner</t>
+          <t>bulkhead / upper</t>
         </is>
       </c>
       <c r="B33" s="15" t="n">
@@ -10627,7 +12195,7 @@
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>driver wall / floor</t>
+          <t>bulkhead corner</t>
         </is>
       </c>
       <c r="B34" s="15" t="n">
@@ -10637,7 +12205,7 @@
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>driver wall / floor / inner</t>
+          <t>driver wall / floor</t>
         </is>
       </c>
       <c r="B35" s="15" t="n">
@@ -10647,7 +12215,7 @@
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>driver wall / upper / inner</t>
+          <t>driver wall / floor / inner</t>
         </is>
       </c>
       <c r="B36" s="15" t="n">
@@ -10657,7 +12225,7 @@
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>floor / bottom corner</t>
+          <t>driver wall / upper / inner</t>
         </is>
       </c>
       <c r="B37" s="15" t="n">
@@ -10667,7 +12235,7 @@
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
         <is>
-          <t>inner / outer corner</t>
+          <t>floor / bottom corner</t>
         </is>
       </c>
       <c r="B38" s="15" t="n">
@@ -10677,7 +12245,7 @@
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>inner corner</t>
+          <t>inner / outer corner</t>
         </is>
       </c>
       <c r="B39" s="15" t="n">
@@ -10687,7 +12255,7 @@
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t>passenger wall / floor</t>
+          <t>inner corner</t>
         </is>
       </c>
       <c r="B40" s="15" t="n">
@@ -10697,7 +12265,7 @@
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>passenger wall / floor / inner</t>
+          <t>passenger wall / floor</t>
         </is>
       </c>
       <c r="B41" s="15" t="n">
@@ -10707,7 +12275,7 @@
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>passenger wall / top / inner</t>
+          <t>passenger wall / floor / inner</t>
         </is>
       </c>
       <c r="B42" s="15" t="n">
@@ -10717,7 +12285,7 @@
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>top / inner</t>
+          <t>passenger wall / top / inner</t>
         </is>
       </c>
       <c r="B43" s="15" t="n">
@@ -10727,7 +12295,7 @@
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
         <is>
-          <t>top / inner corner</t>
+          <t>top / inner</t>
         </is>
       </c>
       <c r="B44" s="15" t="n">
@@ -10737,7 +12305,7 @@
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t>top corner</t>
+          <t>top / inner corner</t>
         </is>
       </c>
       <c r="B45" s="15" t="n">
@@ -10747,10 +12315,20 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>top corner</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>upper</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B47" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>